<commit_message>
Guida: dove trovare i documenti sanitari di famiglia (FSE, vaccini, visite, gruppo sanguigno)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016dnPAsxSX8LqX4WvN5HDSM
</commit_message>
<xml_diff>
--- a/scarica/gestionale-di-famiglia.xlsx
+++ b/scarica/gestionale-di-famiglia.xlsx
@@ -2323,7 +2323,7 @@
         </is>
       </c>
       <c r="C5" s="19" t="n">
-        <v>46332</v>
+        <v>46333</v>
       </c>
       <c r="D5" s="20">
         <f>IF(OR(C5="",F5="☑"),"",C5-TODAY())</f>
@@ -2361,7 +2361,7 @@
         </is>
       </c>
       <c r="C6" s="23" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="D6" s="20">
         <f>IF(OR(C6="",F6="☑"),"",C6-TODAY())</f>
@@ -3103,7 +3103,7 @@
     </row>
     <row r="5" ht="36" customHeight="1">
       <c r="A5" s="19" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="B5" s="18" t="inlineStr">
         <is>
@@ -4211,7 +4211,7 @@
     </row>
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="19" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B5" s="18" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Gestionale: gruppo sanguigno, esenzioni, fascicolo, dati ricetta e disdetta, CUP e URP
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016dnPAsxSX8LqX4WvN5HDSM
</commit_message>
<xml_diff>
--- a/scarica/gestionale-di-famiglia.xlsx
+++ b/scarica/gestionale-di-famiglia.xlsx
@@ -150,7 +150,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -203,6 +203,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -611,7 +614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -702,157 +705,192 @@
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
+          <t>Visite nei prossimi 7 giorni</t>
+        </is>
+      </c>
+      <c r="B10" s="7">
+        <f>COUNTIFS(Visite!A5:A44,"&gt;="&amp;TODAY(),Visite!A5:A44,"&lt;="&amp;(TODAY()+7))</f>
+        <v/>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Scheda Visite: controlla «Disdire entro» e il ticket</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Ticket ancora da pagare</t>
+        </is>
+      </c>
+      <c r="B11" s="7">
+        <f>COUNTIFS(Visite!H5:H44,"Da pagare",Visite!A5:A44,"&gt;="&amp;TODAY())</f>
+        <v/>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Di norma si paga prima della visita</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
           <t>Prossima scadenza tra (giorni)</t>
         </is>
       </c>
-      <c r="B10" s="7">
+      <c r="B12" s="7">
         <f>IF(COUNTIF(Scadenze!D5:D44,"&gt;=0")=0,"—",SUMPRODUCT(MIN(IF(Scadenze!D5:D44&gt;=0,Scadenze!D5:D44))))</f>
         <v/>
       </c>
-      <c r="C10" s="8" t="inlineStr">
+      <c r="C12" s="8" t="inlineStr">
         <is>
           <t>La più vicina tra quelle ancora da fare</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+      <c r="A13" s="5" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>Come si usa</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>Famiglia</t>
-        </is>
-      </c>
-      <c r="C14" s="9" t="inlineStr">
-        <is>
-          <t>Una riga per persona. L'età si calcola da sola.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>Documenti</t>
-        </is>
-      </c>
-      <c r="C15" s="9" t="inlineStr">
-        <is>
-          <t>La cartellina: dove sta ogni documento e quando scade. Lo stato si colora da solo.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Scadenze</t>
+          <t>Famiglia</t>
         </is>
       </c>
       <c r="C16" s="9" t="inlineStr">
         <is>
-          <t>Vaccini, visite, rinnovi, iscrizioni. Spunta "Fatto" e sparisce dai promemoria.</t>
+          <t>Una riga per persona: pediatra, allergie, gruppo sanguigno, esenzioni, stato del Fascicolo sanitario. L'età si calcola da sola.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Visite</t>
+          <t>Documenti</t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>Prima della visita scrivi le domande, la più importante per prima. Dopo, cosa fare e quando richiamare.</t>
+          <t>La cartellina: dove sta ogni documento e quando scade. Lo stato si colora da solo.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Settimana</t>
+          <t>Scadenze</t>
         </is>
       </c>
       <c r="C18" s="9" t="inlineStr">
         <is>
-          <t>La settimana di tutti, con chi se ne occupa: così non ricorda tutto una persona sola.</t>
+          <t>Vaccini, visite, rinnovi, iscrizioni. Spunta "Fatto" e sparisce dai promemoria.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Contatti</t>
+          <t>Visite</t>
         </is>
       </c>
       <c r="C19" s="9" t="inlineStr">
         <is>
-          <t>Pediatra, guardia medica, nido, nonni. Stampalo e mettilo nella cartellina.</t>
+          <t>Ricetta, prenotazione, ticket e la data entro cui disdire senza pagare. Poi le domande, la più importante per prima, e cosa fare dopo.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
+          <t>Settimana</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>La settimana di tutti, con chi se ne occupa: così non ricorda tutto una persona sola.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Contatti</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>Pediatra, guardia medica, nido, nonni. Stampalo e mettilo nella cartellina.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
           <t>Prime volte</t>
         </is>
       </c>
-      <c r="C20" s="9" t="inlineStr">
+      <c r="C22" s="9" t="inlineStr">
         <is>
           <t>I ricordi che non vuoi perdere, scritti il giorno stesso.</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="5" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
         <is>
           <t>Legenda</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="10" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="10" t="inlineStr">
         <is>
           <t>Testo blu su righe alternate</t>
         </is>
       </c>
-      <c r="C23" s="11" t="inlineStr">
+      <c r="C25" s="11" t="inlineStr">
         <is>
           <t>Celle da compilare</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="12" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="12" t="inlineStr">
         <is>
           <t>Testo nero</t>
         </is>
       </c>
-      <c r="C24" s="11" t="inlineStr">
+      <c r="C26" s="11" t="inlineStr">
         <is>
           <t>Si calcola da solo: non scriverci sopra</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="13" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="13" t="inlineStr">
         <is>
           <t>Ogni scheda ha una riga di esempio in grigio: cancellala e scrivi i tuoi dati.</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="30" customHeight="1">
-      <c r="A27" s="14" t="inlineStr">
+    <row r="29" ht="30" customHeight="1">
+      <c r="A29" s="14" t="inlineStr">
         <is>
           <t>Questo file resta sul tuo computer o telefono: nessun dato viene inviato a nessuno. Non sostituisce il pediatra o il medico: per vaccini e terapie il riferimento resta loro.</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="15" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="15" t="inlineStr">
         <is>
           <t>serenainmente.it/guide</t>
         </is>
@@ -860,23 +898,23 @@
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="A25:C25"/>
     <mergeCell ref="A20:B20"/>
+    <mergeCell ref="A21:B21"/>
     <mergeCell ref="A16:B16"/>
-    <mergeCell ref="A15:B15"/>
     <mergeCell ref="A19:B19"/>
     <mergeCell ref="A27:C27"/>
-    <mergeCell ref="A14:B14"/>
     <mergeCell ref="A17:B17"/>
     <mergeCell ref="A18:B18"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A29:C29"/>
   </mergeCells>
-  <conditionalFormatting sqref="B7:B9">
+  <conditionalFormatting sqref="B7:B12">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>B7&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A28" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A30" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -888,7 +926,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H44"/>
+  <dimension ref="A1:K44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -896,9 +934,12 @@
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="28" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -953,6 +994,21 @@
       </c>
       <c r="H4" s="17" t="inlineStr">
         <is>
+          <t>Gruppo sanguigno</t>
+        </is>
+      </c>
+      <c r="I4" s="17" t="inlineStr">
+        <is>
+          <t>Esenzioni (codice)</t>
+        </is>
+      </c>
+      <c r="J4" s="17" t="inlineStr">
+        <is>
+          <t>Fascicolo sanitario</t>
+        </is>
+      </c>
+      <c r="K4" s="17" t="inlineStr">
+        <is>
           <t>Note</t>
         </is>
       </c>
@@ -990,7 +1046,22 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H5" s="21" t="inlineStr">
+      <c r="H5" s="18" t="inlineStr">
+        <is>
+          <t>Non so</t>
+        </is>
+      </c>
+      <c r="I5" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J5" s="18" t="inlineStr">
+        <is>
+          <t>Da attivare (figlio)</t>
+        </is>
+      </c>
+      <c r="K5" s="21" t="inlineStr">
         <is>
           <t>Esempio: cancella questa riga e scrivi i tuoi dati</t>
         </is>
@@ -1008,6 +1079,9 @@
       <c r="F6" s="22" t="n"/>
       <c r="G6" s="22" t="n"/>
       <c r="H6" s="22" t="n"/>
+      <c r="I6" s="22" t="n"/>
+      <c r="J6" s="22" t="n"/>
+      <c r="K6" s="22" t="n"/>
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="18" t="n"/>
@@ -1021,6 +1095,9 @@
       <c r="F7" s="18" t="n"/>
       <c r="G7" s="18" t="n"/>
       <c r="H7" s="18" t="n"/>
+      <c r="I7" s="18" t="n"/>
+      <c r="J7" s="18" t="n"/>
+      <c r="K7" s="18" t="n"/>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="22" t="n"/>
@@ -1034,6 +1111,9 @@
       <c r="F8" s="22" t="n"/>
       <c r="G8" s="22" t="n"/>
       <c r="H8" s="22" t="n"/>
+      <c r="I8" s="22" t="n"/>
+      <c r="J8" s="22" t="n"/>
+      <c r="K8" s="22" t="n"/>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="18" t="n"/>
@@ -1047,6 +1127,9 @@
       <c r="F9" s="18" t="n"/>
       <c r="G9" s="18" t="n"/>
       <c r="H9" s="18" t="n"/>
+      <c r="I9" s="18" t="n"/>
+      <c r="J9" s="18" t="n"/>
+      <c r="K9" s="18" t="n"/>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="22" t="n"/>
@@ -1060,6 +1143,9 @@
       <c r="F10" s="22" t="n"/>
       <c r="G10" s="22" t="n"/>
       <c r="H10" s="22" t="n"/>
+      <c r="I10" s="22" t="n"/>
+      <c r="J10" s="22" t="n"/>
+      <c r="K10" s="22" t="n"/>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="18" t="n"/>
@@ -1073,6 +1159,9 @@
       <c r="F11" s="18" t="n"/>
       <c r="G11" s="18" t="n"/>
       <c r="H11" s="18" t="n"/>
+      <c r="I11" s="18" t="n"/>
+      <c r="J11" s="18" t="n"/>
+      <c r="K11" s="18" t="n"/>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="22" t="n"/>
@@ -1086,6 +1175,9 @@
       <c r="F12" s="22" t="n"/>
       <c r="G12" s="22" t="n"/>
       <c r="H12" s="22" t="n"/>
+      <c r="I12" s="22" t="n"/>
+      <c r="J12" s="22" t="n"/>
+      <c r="K12" s="22" t="n"/>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="18" t="n"/>
@@ -1099,6 +1191,9 @@
       <c r="F13" s="18" t="n"/>
       <c r="G13" s="18" t="n"/>
       <c r="H13" s="18" t="n"/>
+      <c r="I13" s="18" t="n"/>
+      <c r="J13" s="18" t="n"/>
+      <c r="K13" s="18" t="n"/>
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="22" t="n"/>
@@ -1112,6 +1207,9 @@
       <c r="F14" s="22" t="n"/>
       <c r="G14" s="22" t="n"/>
       <c r="H14" s="22" t="n"/>
+      <c r="I14" s="22" t="n"/>
+      <c r="J14" s="22" t="n"/>
+      <c r="K14" s="22" t="n"/>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="18" t="n"/>
@@ -1125,6 +1223,9 @@
       <c r="F15" s="18" t="n"/>
       <c r="G15" s="18" t="n"/>
       <c r="H15" s="18" t="n"/>
+      <c r="I15" s="18" t="n"/>
+      <c r="J15" s="18" t="n"/>
+      <c r="K15" s="18" t="n"/>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="22" t="n"/>
@@ -1138,6 +1239,9 @@
       <c r="F16" s="22" t="n"/>
       <c r="G16" s="22" t="n"/>
       <c r="H16" s="22" t="n"/>
+      <c r="I16" s="22" t="n"/>
+      <c r="J16" s="22" t="n"/>
+      <c r="K16" s="22" t="n"/>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="18" t="n"/>
@@ -1151,6 +1255,9 @@
       <c r="F17" s="18" t="n"/>
       <c r="G17" s="18" t="n"/>
       <c r="H17" s="18" t="n"/>
+      <c r="I17" s="18" t="n"/>
+      <c r="J17" s="18" t="n"/>
+      <c r="K17" s="18" t="n"/>
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="22" t="n"/>
@@ -1164,6 +1271,9 @@
       <c r="F18" s="22" t="n"/>
       <c r="G18" s="22" t="n"/>
       <c r="H18" s="22" t="n"/>
+      <c r="I18" s="22" t="n"/>
+      <c r="J18" s="22" t="n"/>
+      <c r="K18" s="22" t="n"/>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="18" t="n"/>
@@ -1177,6 +1287,9 @@
       <c r="F19" s="18" t="n"/>
       <c r="G19" s="18" t="n"/>
       <c r="H19" s="18" t="n"/>
+      <c r="I19" s="18" t="n"/>
+      <c r="J19" s="18" t="n"/>
+      <c r="K19" s="18" t="n"/>
     </row>
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="22" t="n"/>
@@ -1190,6 +1303,9 @@
       <c r="F20" s="22" t="n"/>
       <c r="G20" s="22" t="n"/>
       <c r="H20" s="22" t="n"/>
+      <c r="I20" s="22" t="n"/>
+      <c r="J20" s="22" t="n"/>
+      <c r="K20" s="22" t="n"/>
     </row>
     <row r="21" ht="20" customHeight="1">
       <c r="A21" s="18" t="n"/>
@@ -1203,6 +1319,9 @@
       <c r="F21" s="18" t="n"/>
       <c r="G21" s="18" t="n"/>
       <c r="H21" s="18" t="n"/>
+      <c r="I21" s="18" t="n"/>
+      <c r="J21" s="18" t="n"/>
+      <c r="K21" s="18" t="n"/>
     </row>
     <row r="22" ht="20" customHeight="1">
       <c r="A22" s="22" t="n"/>
@@ -1216,6 +1335,9 @@
       <c r="F22" s="22" t="n"/>
       <c r="G22" s="22" t="n"/>
       <c r="H22" s="22" t="n"/>
+      <c r="I22" s="22" t="n"/>
+      <c r="J22" s="22" t="n"/>
+      <c r="K22" s="22" t="n"/>
     </row>
     <row r="23" ht="20" customHeight="1">
       <c r="A23" s="18" t="n"/>
@@ -1229,6 +1351,9 @@
       <c r="F23" s="18" t="n"/>
       <c r="G23" s="18" t="n"/>
       <c r="H23" s="18" t="n"/>
+      <c r="I23" s="18" t="n"/>
+      <c r="J23" s="18" t="n"/>
+      <c r="K23" s="18" t="n"/>
     </row>
     <row r="24" ht="20" customHeight="1">
       <c r="A24" s="22" t="n"/>
@@ -1242,6 +1367,9 @@
       <c r="F24" s="22" t="n"/>
       <c r="G24" s="22" t="n"/>
       <c r="H24" s="22" t="n"/>
+      <c r="I24" s="22" t="n"/>
+      <c r="J24" s="22" t="n"/>
+      <c r="K24" s="22" t="n"/>
     </row>
     <row r="25" ht="20" customHeight="1">
       <c r="A25" s="18" t="n"/>
@@ -1255,6 +1383,9 @@
       <c r="F25" s="18" t="n"/>
       <c r="G25" s="18" t="n"/>
       <c r="H25" s="18" t="n"/>
+      <c r="I25" s="18" t="n"/>
+      <c r="J25" s="18" t="n"/>
+      <c r="K25" s="18" t="n"/>
     </row>
     <row r="26" ht="20" customHeight="1">
       <c r="A26" s="22" t="n"/>
@@ -1268,6 +1399,9 @@
       <c r="F26" s="22" t="n"/>
       <c r="G26" s="22" t="n"/>
       <c r="H26" s="22" t="n"/>
+      <c r="I26" s="22" t="n"/>
+      <c r="J26" s="22" t="n"/>
+      <c r="K26" s="22" t="n"/>
     </row>
     <row r="27" ht="20" customHeight="1">
       <c r="A27" s="18" t="n"/>
@@ -1281,6 +1415,9 @@
       <c r="F27" s="18" t="n"/>
       <c r="G27" s="18" t="n"/>
       <c r="H27" s="18" t="n"/>
+      <c r="I27" s="18" t="n"/>
+      <c r="J27" s="18" t="n"/>
+      <c r="K27" s="18" t="n"/>
     </row>
     <row r="28" ht="20" customHeight="1">
       <c r="A28" s="22" t="n"/>
@@ -1294,6 +1431,9 @@
       <c r="F28" s="22" t="n"/>
       <c r="G28" s="22" t="n"/>
       <c r="H28" s="22" t="n"/>
+      <c r="I28" s="22" t="n"/>
+      <c r="J28" s="22" t="n"/>
+      <c r="K28" s="22" t="n"/>
     </row>
     <row r="29" ht="20" customHeight="1">
       <c r="A29" s="18" t="n"/>
@@ -1307,6 +1447,9 @@
       <c r="F29" s="18" t="n"/>
       <c r="G29" s="18" t="n"/>
       <c r="H29" s="18" t="n"/>
+      <c r="I29" s="18" t="n"/>
+      <c r="J29" s="18" t="n"/>
+      <c r="K29" s="18" t="n"/>
     </row>
     <row r="30" ht="20" customHeight="1">
       <c r="A30" s="22" t="n"/>
@@ -1320,6 +1463,9 @@
       <c r="F30" s="22" t="n"/>
       <c r="G30" s="22" t="n"/>
       <c r="H30" s="22" t="n"/>
+      <c r="I30" s="22" t="n"/>
+      <c r="J30" s="22" t="n"/>
+      <c r="K30" s="22" t="n"/>
     </row>
     <row r="31" ht="20" customHeight="1">
       <c r="A31" s="18" t="n"/>
@@ -1333,6 +1479,9 @@
       <c r="F31" s="18" t="n"/>
       <c r="G31" s="18" t="n"/>
       <c r="H31" s="18" t="n"/>
+      <c r="I31" s="18" t="n"/>
+      <c r="J31" s="18" t="n"/>
+      <c r="K31" s="18" t="n"/>
     </row>
     <row r="32" ht="20" customHeight="1">
       <c r="A32" s="22" t="n"/>
@@ -1346,6 +1495,9 @@
       <c r="F32" s="22" t="n"/>
       <c r="G32" s="22" t="n"/>
       <c r="H32" s="22" t="n"/>
+      <c r="I32" s="22" t="n"/>
+      <c r="J32" s="22" t="n"/>
+      <c r="K32" s="22" t="n"/>
     </row>
     <row r="33" ht="20" customHeight="1">
       <c r="A33" s="18" t="n"/>
@@ -1359,6 +1511,9 @@
       <c r="F33" s="18" t="n"/>
       <c r="G33" s="18" t="n"/>
       <c r="H33" s="18" t="n"/>
+      <c r="I33" s="18" t="n"/>
+      <c r="J33" s="18" t="n"/>
+      <c r="K33" s="18" t="n"/>
     </row>
     <row r="34" ht="20" customHeight="1">
       <c r="A34" s="22" t="n"/>
@@ -1372,6 +1527,9 @@
       <c r="F34" s="22" t="n"/>
       <c r="G34" s="22" t="n"/>
       <c r="H34" s="22" t="n"/>
+      <c r="I34" s="22" t="n"/>
+      <c r="J34" s="22" t="n"/>
+      <c r="K34" s="22" t="n"/>
     </row>
     <row r="35" ht="20" customHeight="1">
       <c r="A35" s="18" t="n"/>
@@ -1385,6 +1543,9 @@
       <c r="F35" s="18" t="n"/>
       <c r="G35" s="18" t="n"/>
       <c r="H35" s="18" t="n"/>
+      <c r="I35" s="18" t="n"/>
+      <c r="J35" s="18" t="n"/>
+      <c r="K35" s="18" t="n"/>
     </row>
     <row r="36" ht="20" customHeight="1">
       <c r="A36" s="22" t="n"/>
@@ -1398,6 +1559,9 @@
       <c r="F36" s="22" t="n"/>
       <c r="G36" s="22" t="n"/>
       <c r="H36" s="22" t="n"/>
+      <c r="I36" s="22" t="n"/>
+      <c r="J36" s="22" t="n"/>
+      <c r="K36" s="22" t="n"/>
     </row>
     <row r="37" ht="20" customHeight="1">
       <c r="A37" s="18" t="n"/>
@@ -1411,6 +1575,9 @@
       <c r="F37" s="18" t="n"/>
       <c r="G37" s="18" t="n"/>
       <c r="H37" s="18" t="n"/>
+      <c r="I37" s="18" t="n"/>
+      <c r="J37" s="18" t="n"/>
+      <c r="K37" s="18" t="n"/>
     </row>
     <row r="38" ht="20" customHeight="1">
       <c r="A38" s="22" t="n"/>
@@ -1424,6 +1591,9 @@
       <c r="F38" s="22" t="n"/>
       <c r="G38" s="22" t="n"/>
       <c r="H38" s="22" t="n"/>
+      <c r="I38" s="22" t="n"/>
+      <c r="J38" s="22" t="n"/>
+      <c r="K38" s="22" t="n"/>
     </row>
     <row r="39" ht="20" customHeight="1">
       <c r="A39" s="18" t="n"/>
@@ -1437,6 +1607,9 @@
       <c r="F39" s="18" t="n"/>
       <c r="G39" s="18" t="n"/>
       <c r="H39" s="18" t="n"/>
+      <c r="I39" s="18" t="n"/>
+      <c r="J39" s="18" t="n"/>
+      <c r="K39" s="18" t="n"/>
     </row>
     <row r="40" ht="20" customHeight="1">
       <c r="A40" s="22" t="n"/>
@@ -1450,6 +1623,9 @@
       <c r="F40" s="22" t="n"/>
       <c r="G40" s="22" t="n"/>
       <c r="H40" s="22" t="n"/>
+      <c r="I40" s="22" t="n"/>
+      <c r="J40" s="22" t="n"/>
+      <c r="K40" s="22" t="n"/>
     </row>
     <row r="41" ht="20" customHeight="1">
       <c r="A41" s="18" t="n"/>
@@ -1463,6 +1639,9 @@
       <c r="F41" s="18" t="n"/>
       <c r="G41" s="18" t="n"/>
       <c r="H41" s="18" t="n"/>
+      <c r="I41" s="18" t="n"/>
+      <c r="J41" s="18" t="n"/>
+      <c r="K41" s="18" t="n"/>
     </row>
     <row r="42" ht="20" customHeight="1">
       <c r="A42" s="22" t="n"/>
@@ -1476,6 +1655,9 @@
       <c r="F42" s="22" t="n"/>
       <c r="G42" s="22" t="n"/>
       <c r="H42" s="22" t="n"/>
+      <c r="I42" s="22" t="n"/>
+      <c r="J42" s="22" t="n"/>
+      <c r="K42" s="22" t="n"/>
     </row>
     <row r="43" ht="20" customHeight="1">
       <c r="A43" s="18" t="n"/>
@@ -1489,6 +1671,9 @@
       <c r="F43" s="18" t="n"/>
       <c r="G43" s="18" t="n"/>
       <c r="H43" s="18" t="n"/>
+      <c r="I43" s="18" t="n"/>
+      <c r="J43" s="18" t="n"/>
+      <c r="K43" s="18" t="n"/>
     </row>
     <row r="44" ht="20" customHeight="1">
       <c r="A44" s="22" t="n"/>
@@ -1502,9 +1687,18 @@
       <c r="F44" s="22" t="n"/>
       <c r="G44" s="22" t="n"/>
       <c r="H44" s="22" t="n"/>
+      <c r="I44" s="22" t="n"/>
+      <c r="J44" s="22" t="n"/>
+      <c r="K44" s="22" t="n"/>
     </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations count="3">
+    <dataValidation sqref="H5 H6 H7 H8 H9 H10 H11 H12 H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H25 H26 H27 H28 H29 H30 H31 H32 H33 H34 H35 H36 H37 H38 H39 H40 H41 H42 H43 H44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Non so,0+,0-,A+,A-,B+,B-,AB+,AB-"</formula1>
+    </dataValidation>
+    <dataValidation sqref="J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J20 J21 J22 J23 J24 J25 J26 J27 J28 J29 J30 J31 J32 J33 J34 J35 J36 J37 J38 J39 J40 J41 J42 J43 J44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Attivo, consenso dato,Attivo, consenso da dare,Da attivare (figlio),Non so"</formula1>
+    </dataValidation>
     <dataValidation sqref="B5 B6 B7 B8 B9 B10 B11 B12 B13 B14 B15 B16 B17 B18 B19 B20 B21 B22 B23 B24 B25 B26 B27 B28 B29 B30 B31 B32 B33 B34 B35 B36 B37 B38 B39 B40 B41 B42 B43 B44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Mamma,Papà,Bambino/a,Nonno/a,Altro"</formula1>
     </dataValidation>
@@ -1520,16 +1714,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G44"/>
+  <dimension ref="A1:H44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="9" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -1559,7 +1754,7 @@
       </c>
       <c r="C4" s="17" t="inlineStr">
         <is>
-          <t>Dove si trova</t>
+          <t>Dove si trova (carta)</t>
         </is>
       </c>
       <c r="D4" s="17" t="inlineStr">
@@ -1578,6 +1773,11 @@
         </is>
       </c>
       <c r="G4" s="17" t="inlineStr">
+        <is>
+          <t>Dove sta online</t>
+        </is>
+      </c>
+      <c r="H4" s="17" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
@@ -1610,7 +1810,12 @@
         <f>IF(D5="","",IF(E5&lt;0,"Scaduto",IF(E5&lt;=30,"In scadenza","Ok")))</f>
         <v/>
       </c>
-      <c r="G5" s="21" t="inlineStr">
+      <c r="G5" s="18" t="inlineStr">
+        <is>
+          <t>App IO</t>
+        </is>
+      </c>
+      <c r="H5" s="21" t="inlineStr">
         <is>
           <t>Esempio: cancella questa riga e scrivi i tuoi dati</t>
         </is>
@@ -1641,7 +1846,12 @@
         <f>IF(D6="","",IF(E6&lt;0,"Scaduto",IF(E6&lt;=30,"In scadenza","Ok")))</f>
         <v/>
       </c>
-      <c r="G6" s="24" t="inlineStr">
+      <c r="G6" s="22" t="inlineStr">
+        <is>
+          <t>Fascicolo sanitario</t>
+        </is>
+      </c>
+      <c r="H6" s="24" t="inlineStr">
         <is>
           <t>Senza scadenza: lascia vuota la data</t>
         </is>
@@ -1661,6 +1871,7 @@
         <v/>
       </c>
       <c r="G7" s="18" t="n"/>
+      <c r="H7" s="18" t="n"/>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="22" t="n"/>
@@ -1676,6 +1887,7 @@
         <v/>
       </c>
       <c r="G8" s="22" t="n"/>
+      <c r="H8" s="22" t="n"/>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="18" t="n"/>
@@ -1691,6 +1903,7 @@
         <v/>
       </c>
       <c r="G9" s="18" t="n"/>
+      <c r="H9" s="18" t="n"/>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="22" t="n"/>
@@ -1706,6 +1919,7 @@
         <v/>
       </c>
       <c r="G10" s="22" t="n"/>
+      <c r="H10" s="22" t="n"/>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="18" t="n"/>
@@ -1721,6 +1935,7 @@
         <v/>
       </c>
       <c r="G11" s="18" t="n"/>
+      <c r="H11" s="18" t="n"/>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="22" t="n"/>
@@ -1736,6 +1951,7 @@
         <v/>
       </c>
       <c r="G12" s="22" t="n"/>
+      <c r="H12" s="22" t="n"/>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="18" t="n"/>
@@ -1751,6 +1967,7 @@
         <v/>
       </c>
       <c r="G13" s="18" t="n"/>
+      <c r="H13" s="18" t="n"/>
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="22" t="n"/>
@@ -1766,6 +1983,7 @@
         <v/>
       </c>
       <c r="G14" s="22" t="n"/>
+      <c r="H14" s="22" t="n"/>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="18" t="n"/>
@@ -1781,6 +1999,7 @@
         <v/>
       </c>
       <c r="G15" s="18" t="n"/>
+      <c r="H15" s="18" t="n"/>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="22" t="n"/>
@@ -1796,6 +2015,7 @@
         <v/>
       </c>
       <c r="G16" s="22" t="n"/>
+      <c r="H16" s="22" t="n"/>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="18" t="n"/>
@@ -1811,6 +2031,7 @@
         <v/>
       </c>
       <c r="G17" s="18" t="n"/>
+      <c r="H17" s="18" t="n"/>
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="22" t="n"/>
@@ -1826,6 +2047,7 @@
         <v/>
       </c>
       <c r="G18" s="22" t="n"/>
+      <c r="H18" s="22" t="n"/>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="18" t="n"/>
@@ -1841,6 +2063,7 @@
         <v/>
       </c>
       <c r="G19" s="18" t="n"/>
+      <c r="H19" s="18" t="n"/>
     </row>
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="22" t="n"/>
@@ -1856,6 +2079,7 @@
         <v/>
       </c>
       <c r="G20" s="22" t="n"/>
+      <c r="H20" s="22" t="n"/>
     </row>
     <row r="21" ht="20" customHeight="1">
       <c r="A21" s="18" t="n"/>
@@ -1871,6 +2095,7 @@
         <v/>
       </c>
       <c r="G21" s="18" t="n"/>
+      <c r="H21" s="18" t="n"/>
     </row>
     <row r="22" ht="20" customHeight="1">
       <c r="A22" s="22" t="n"/>
@@ -1886,6 +2111,7 @@
         <v/>
       </c>
       <c r="G22" s="22" t="n"/>
+      <c r="H22" s="22" t="n"/>
     </row>
     <row r="23" ht="20" customHeight="1">
       <c r="A23" s="18" t="n"/>
@@ -1901,6 +2127,7 @@
         <v/>
       </c>
       <c r="G23" s="18" t="n"/>
+      <c r="H23" s="18" t="n"/>
     </row>
     <row r="24" ht="20" customHeight="1">
       <c r="A24" s="22" t="n"/>
@@ -1916,6 +2143,7 @@
         <v/>
       </c>
       <c r="G24" s="22" t="n"/>
+      <c r="H24" s="22" t="n"/>
     </row>
     <row r="25" ht="20" customHeight="1">
       <c r="A25" s="18" t="n"/>
@@ -1931,6 +2159,7 @@
         <v/>
       </c>
       <c r="G25" s="18" t="n"/>
+      <c r="H25" s="18" t="n"/>
     </row>
     <row r="26" ht="20" customHeight="1">
       <c r="A26" s="22" t="n"/>
@@ -1946,6 +2175,7 @@
         <v/>
       </c>
       <c r="G26" s="22" t="n"/>
+      <c r="H26" s="22" t="n"/>
     </row>
     <row r="27" ht="20" customHeight="1">
       <c r="A27" s="18" t="n"/>
@@ -1961,6 +2191,7 @@
         <v/>
       </c>
       <c r="G27" s="18" t="n"/>
+      <c r="H27" s="18" t="n"/>
     </row>
     <row r="28" ht="20" customHeight="1">
       <c r="A28" s="22" t="n"/>
@@ -1976,6 +2207,7 @@
         <v/>
       </c>
       <c r="G28" s="22" t="n"/>
+      <c r="H28" s="22" t="n"/>
     </row>
     <row r="29" ht="20" customHeight="1">
       <c r="A29" s="18" t="n"/>
@@ -1991,6 +2223,7 @@
         <v/>
       </c>
       <c r="G29" s="18" t="n"/>
+      <c r="H29" s="18" t="n"/>
     </row>
     <row r="30" ht="20" customHeight="1">
       <c r="A30" s="22" t="n"/>
@@ -2006,6 +2239,7 @@
         <v/>
       </c>
       <c r="G30" s="22" t="n"/>
+      <c r="H30" s="22" t="n"/>
     </row>
     <row r="31" ht="20" customHeight="1">
       <c r="A31" s="18" t="n"/>
@@ -2021,6 +2255,7 @@
         <v/>
       </c>
       <c r="G31" s="18" t="n"/>
+      <c r="H31" s="18" t="n"/>
     </row>
     <row r="32" ht="20" customHeight="1">
       <c r="A32" s="22" t="n"/>
@@ -2036,6 +2271,7 @@
         <v/>
       </c>
       <c r="G32" s="22" t="n"/>
+      <c r="H32" s="22" t="n"/>
     </row>
     <row r="33" ht="20" customHeight="1">
       <c r="A33" s="18" t="n"/>
@@ -2051,6 +2287,7 @@
         <v/>
       </c>
       <c r="G33" s="18" t="n"/>
+      <c r="H33" s="18" t="n"/>
     </row>
     <row r="34" ht="20" customHeight="1">
       <c r="A34" s="22" t="n"/>
@@ -2066,6 +2303,7 @@
         <v/>
       </c>
       <c r="G34" s="22" t="n"/>
+      <c r="H34" s="22" t="n"/>
     </row>
     <row r="35" ht="20" customHeight="1">
       <c r="A35" s="18" t="n"/>
@@ -2081,6 +2319,7 @@
         <v/>
       </c>
       <c r="G35" s="18" t="n"/>
+      <c r="H35" s="18" t="n"/>
     </row>
     <row r="36" ht="20" customHeight="1">
       <c r="A36" s="22" t="n"/>
@@ -2096,6 +2335,7 @@
         <v/>
       </c>
       <c r="G36" s="22" t="n"/>
+      <c r="H36" s="22" t="n"/>
     </row>
     <row r="37" ht="20" customHeight="1">
       <c r="A37" s="18" t="n"/>
@@ -2111,6 +2351,7 @@
         <v/>
       </c>
       <c r="G37" s="18" t="n"/>
+      <c r="H37" s="18" t="n"/>
     </row>
     <row r="38" ht="20" customHeight="1">
       <c r="A38" s="22" t="n"/>
@@ -2126,6 +2367,7 @@
         <v/>
       </c>
       <c r="G38" s="22" t="n"/>
+      <c r="H38" s="22" t="n"/>
     </row>
     <row r="39" ht="20" customHeight="1">
       <c r="A39" s="18" t="n"/>
@@ -2141,6 +2383,7 @@
         <v/>
       </c>
       <c r="G39" s="18" t="n"/>
+      <c r="H39" s="18" t="n"/>
     </row>
     <row r="40" ht="20" customHeight="1">
       <c r="A40" s="22" t="n"/>
@@ -2156,6 +2399,7 @@
         <v/>
       </c>
       <c r="G40" s="22" t="n"/>
+      <c r="H40" s="22" t="n"/>
     </row>
     <row r="41" ht="20" customHeight="1">
       <c r="A41" s="18" t="n"/>
@@ -2171,6 +2415,7 @@
         <v/>
       </c>
       <c r="G41" s="18" t="n"/>
+      <c r="H41" s="18" t="n"/>
     </row>
     <row r="42" ht="20" customHeight="1">
       <c r="A42" s="22" t="n"/>
@@ -2186,6 +2431,7 @@
         <v/>
       </c>
       <c r="G42" s="22" t="n"/>
+      <c r="H42" s="22" t="n"/>
     </row>
     <row r="43" ht="20" customHeight="1">
       <c r="A43" s="18" t="n"/>
@@ -2201,6 +2447,7 @@
         <v/>
       </c>
       <c r="G43" s="18" t="n"/>
+      <c r="H43" s="18" t="n"/>
     </row>
     <row r="44" ht="20" customHeight="1">
       <c r="A44" s="22" t="n"/>
@@ -2216,6 +2463,7 @@
         <v/>
       </c>
       <c r="G44" s="22" t="n"/>
+      <c r="H44" s="22" t="n"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="F5:F44">
@@ -2226,7 +2474,10 @@
       <formula>AND(ISNUMBER(E5),E5&gt;=0,E5&lt;=30)</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="1">
+  <dataValidations count="2">
+    <dataValidation sqref="G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G25 G26 G27 G28 G29 G30 G31 G32 G33 G34 G35 G36 G37 G38 G39 G40 G41 G42 G43 G44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Fascicolo sanitario,App IO,Mail,Foto sul telefono,Da nessuna parte"</formula1>
+    </dataValidation>
     <dataValidation sqref="A5 A6 A7 A8 A9 A10 A11 A12 A13 A14 A15 A16 A17 A18 A19 A20 A21 A22 A23 A24 A25 A26 A27 A28 A29 A30 A31 A32 A33 A34 A35 A36 A37 A38 A39 A40 A41 A42 A43 A44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Tessera sanitaria,Carta d'identità,Passaporto,Libretto vaccinale,Referto,Lettera di dimissione,Certificato,Altro"</formula1>
     </dataValidation>
@@ -3020,19 +3271,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J44"/>
+  <dimension ref="A1:O44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="26" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
     <col width="26" customWidth="1" min="9" max="9"/>
     <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="26" customWidth="1" min="12" max="12"/>
+    <col width="30" customWidth="1" min="13" max="13"/>
+    <col width="26" customWidth="1" min="14" max="14"/>
+    <col width="22" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -3045,7 +3301,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Dieci minuti prima: scrivi le domande e cosa hai notato. Durante: le risposte. Prima di uscire: cosa fare e quando richiamare.</t>
+          <t>Ricetta, prenotazione e ticket in alto; domande e risposte a seguire. "Disdire entro" si calcola da solo (due giorni lavorativi prima).</t>
         </is>
       </c>
     </row>
@@ -3062,40 +3318,65 @@
       </c>
       <c r="C4" s="17" t="inlineStr">
         <is>
-          <t>Medico</t>
+          <t>Medico / struttura</t>
         </is>
       </c>
       <c r="D4" s="17" t="inlineStr">
         <is>
+          <t>Priorità ricetta</t>
+        </is>
+      </c>
+      <c r="E4" s="17" t="inlineStr">
+        <is>
+          <t>Scadenza ricetta</t>
+        </is>
+      </c>
+      <c r="F4" s="17" t="inlineStr">
+        <is>
+          <t>N. prenotazione</t>
+        </is>
+      </c>
+      <c r="G4" s="17" t="inlineStr">
+        <is>
+          <t>Disdire entro</t>
+        </is>
+      </c>
+      <c r="H4" s="17" t="inlineStr">
+        <is>
+          <t>Ticket</t>
+        </is>
+      </c>
+      <c r="I4" s="17" t="inlineStr">
+        <is>
           <t>Domanda 1 (la più importante)</t>
         </is>
       </c>
-      <c r="E4" s="17" t="inlineStr">
+      <c r="J4" s="17" t="inlineStr">
         <is>
           <t>Domanda 2</t>
         </is>
       </c>
-      <c r="F4" s="17" t="inlineStr">
+      <c r="K4" s="17" t="inlineStr">
         <is>
           <t>Domanda 3</t>
         </is>
       </c>
-      <c r="G4" s="17" t="inlineStr">
+      <c r="L4" s="17" t="inlineStr">
         <is>
           <t>Cosa ho notato</t>
         </is>
       </c>
-      <c r="H4" s="17" t="inlineStr">
+      <c r="M4" s="17" t="inlineStr">
         <is>
           <t>Risposte</t>
         </is>
       </c>
-      <c r="I4" s="17" t="inlineStr">
+      <c r="N4" s="17" t="inlineStr">
         <is>
           <t>Cosa facciamo</t>
         </is>
       </c>
-      <c r="J4" s="17" t="inlineStr">
+      <c r="O4" s="17" t="inlineStr">
         <is>
           <t>Richiamare se / quando</t>
         </is>
@@ -3112,32 +3393,54 @@
       </c>
       <c r="C5" s="18" t="inlineStr">
         <is>
-          <t>Dott.ssa Rossi</t>
+          <t>Dott.ssa Rossi · Osp. Gaslini</t>
         </is>
       </c>
       <c r="D5" s="18" t="inlineStr">
         <is>
+          <t>D (30/60 giorni)</t>
+        </is>
+      </c>
+      <c r="E5" s="19" t="n">
+        <v>46612</v>
+      </c>
+      <c r="F5" s="18" t="inlineStr">
+        <is>
+          <t>CUP 12345678</t>
+        </is>
+      </c>
+      <c r="G5" s="27">
+        <f>IF(A5="","",WORKDAY(A5,-2))</f>
+        <v/>
+      </c>
+      <c r="H5" s="18" t="inlineStr">
+        <is>
+          <t>Da pagare</t>
+        </is>
+      </c>
+      <c r="I5" s="18" t="inlineStr">
+        <is>
           <t>Si sveglia 3 volte a notte: è normale a questa età?</t>
         </is>
       </c>
-      <c r="E5" s="18" t="inlineStr">
+      <c r="J5" s="18" t="inlineStr">
         <is>
           <t>Mangia poco a cena</t>
         </is>
       </c>
-      <c r="F5" s="18" t="inlineStr">
+      <c r="K5" s="18" t="inlineStr">
         <is>
           <t>Quando il prossimo richiamo?</t>
         </is>
       </c>
-      <c r="G5" s="18" t="inlineStr">
+      <c r="L5" s="18" t="inlineStr">
         <is>
           <t>Da due settimane, soprattutto dopo giornate al nido</t>
         </is>
       </c>
-      <c r="H5" s="18" t="inlineStr"/>
-      <c r="I5" s="18" t="inlineStr"/>
-      <c r="J5" s="21" t="inlineStr">
+      <c r="M5" s="18" t="inlineStr"/>
+      <c r="N5" s="18" t="inlineStr"/>
+      <c r="O5" s="21" t="inlineStr">
         <is>
           <t>Esempio: cancella questa riga e scrivi i tuoi dati</t>
         </is>
@@ -3148,470 +3451,795 @@
       <c r="B6" s="22" t="n"/>
       <c r="C6" s="22" t="n"/>
       <c r="D6" s="22" t="n"/>
-      <c r="E6" s="22" t="n"/>
+      <c r="E6" s="23" t="n"/>
       <c r="F6" s="22" t="n"/>
-      <c r="G6" s="22" t="n"/>
+      <c r="G6" s="27">
+        <f>IF(A6="","",WORKDAY(A6,-2))</f>
+        <v/>
+      </c>
       <c r="H6" s="22" t="n"/>
       <c r="I6" s="22" t="n"/>
       <c r="J6" s="22" t="n"/>
+      <c r="K6" s="22" t="n"/>
+      <c r="L6" s="22" t="n"/>
+      <c r="M6" s="22" t="n"/>
+      <c r="N6" s="22" t="n"/>
+      <c r="O6" s="22" t="n"/>
     </row>
     <row r="7" ht="36" customHeight="1">
       <c r="A7" s="19" t="n"/>
       <c r="B7" s="18" t="n"/>
       <c r="C7" s="18" t="n"/>
       <c r="D7" s="18" t="n"/>
-      <c r="E7" s="18" t="n"/>
+      <c r="E7" s="19" t="n"/>
       <c r="F7" s="18" t="n"/>
-      <c r="G7" s="18" t="n"/>
+      <c r="G7" s="27">
+        <f>IF(A7="","",WORKDAY(A7,-2))</f>
+        <v/>
+      </c>
       <c r="H7" s="18" t="n"/>
       <c r="I7" s="18" t="n"/>
       <c r="J7" s="18" t="n"/>
+      <c r="K7" s="18" t="n"/>
+      <c r="L7" s="18" t="n"/>
+      <c r="M7" s="18" t="n"/>
+      <c r="N7" s="18" t="n"/>
+      <c r="O7" s="18" t="n"/>
     </row>
     <row r="8" ht="36" customHeight="1">
       <c r="A8" s="23" t="n"/>
       <c r="B8" s="22" t="n"/>
       <c r="C8" s="22" t="n"/>
       <c r="D8" s="22" t="n"/>
-      <c r="E8" s="22" t="n"/>
+      <c r="E8" s="23" t="n"/>
       <c r="F8" s="22" t="n"/>
-      <c r="G8" s="22" t="n"/>
+      <c r="G8" s="27">
+        <f>IF(A8="","",WORKDAY(A8,-2))</f>
+        <v/>
+      </c>
       <c r="H8" s="22" t="n"/>
       <c r="I8" s="22" t="n"/>
       <c r="J8" s="22" t="n"/>
+      <c r="K8" s="22" t="n"/>
+      <c r="L8" s="22" t="n"/>
+      <c r="M8" s="22" t="n"/>
+      <c r="N8" s="22" t="n"/>
+      <c r="O8" s="22" t="n"/>
     </row>
     <row r="9" ht="36" customHeight="1">
       <c r="A9" s="19" t="n"/>
       <c r="B9" s="18" t="n"/>
       <c r="C9" s="18" t="n"/>
       <c r="D9" s="18" t="n"/>
-      <c r="E9" s="18" t="n"/>
+      <c r="E9" s="19" t="n"/>
       <c r="F9" s="18" t="n"/>
-      <c r="G9" s="18" t="n"/>
+      <c r="G9" s="27">
+        <f>IF(A9="","",WORKDAY(A9,-2))</f>
+        <v/>
+      </c>
       <c r="H9" s="18" t="n"/>
       <c r="I9" s="18" t="n"/>
       <c r="J9" s="18" t="n"/>
+      <c r="K9" s="18" t="n"/>
+      <c r="L9" s="18" t="n"/>
+      <c r="M9" s="18" t="n"/>
+      <c r="N9" s="18" t="n"/>
+      <c r="O9" s="18" t="n"/>
     </row>
     <row r="10" ht="36" customHeight="1">
       <c r="A10" s="23" t="n"/>
       <c r="B10" s="22" t="n"/>
       <c r="C10" s="22" t="n"/>
       <c r="D10" s="22" t="n"/>
-      <c r="E10" s="22" t="n"/>
+      <c r="E10" s="23" t="n"/>
       <c r="F10" s="22" t="n"/>
-      <c r="G10" s="22" t="n"/>
+      <c r="G10" s="27">
+        <f>IF(A10="","",WORKDAY(A10,-2))</f>
+        <v/>
+      </c>
       <c r="H10" s="22" t="n"/>
       <c r="I10" s="22" t="n"/>
       <c r="J10" s="22" t="n"/>
+      <c r="K10" s="22" t="n"/>
+      <c r="L10" s="22" t="n"/>
+      <c r="M10" s="22" t="n"/>
+      <c r="N10" s="22" t="n"/>
+      <c r="O10" s="22" t="n"/>
     </row>
     <row r="11" ht="36" customHeight="1">
       <c r="A11" s="19" t="n"/>
       <c r="B11" s="18" t="n"/>
       <c r="C11" s="18" t="n"/>
       <c r="D11" s="18" t="n"/>
-      <c r="E11" s="18" t="n"/>
+      <c r="E11" s="19" t="n"/>
       <c r="F11" s="18" t="n"/>
-      <c r="G11" s="18" t="n"/>
+      <c r="G11" s="27">
+        <f>IF(A11="","",WORKDAY(A11,-2))</f>
+        <v/>
+      </c>
       <c r="H11" s="18" t="n"/>
       <c r="I11" s="18" t="n"/>
       <c r="J11" s="18" t="n"/>
+      <c r="K11" s="18" t="n"/>
+      <c r="L11" s="18" t="n"/>
+      <c r="M11" s="18" t="n"/>
+      <c r="N11" s="18" t="n"/>
+      <c r="O11" s="18" t="n"/>
     </row>
     <row r="12" ht="36" customHeight="1">
       <c r="A12" s="23" t="n"/>
       <c r="B12" s="22" t="n"/>
       <c r="C12" s="22" t="n"/>
       <c r="D12" s="22" t="n"/>
-      <c r="E12" s="22" t="n"/>
+      <c r="E12" s="23" t="n"/>
       <c r="F12" s="22" t="n"/>
-      <c r="G12" s="22" t="n"/>
+      <c r="G12" s="27">
+        <f>IF(A12="","",WORKDAY(A12,-2))</f>
+        <v/>
+      </c>
       <c r="H12" s="22" t="n"/>
       <c r="I12" s="22" t="n"/>
       <c r="J12" s="22" t="n"/>
+      <c r="K12" s="22" t="n"/>
+      <c r="L12" s="22" t="n"/>
+      <c r="M12" s="22" t="n"/>
+      <c r="N12" s="22" t="n"/>
+      <c r="O12" s="22" t="n"/>
     </row>
     <row r="13" ht="36" customHeight="1">
       <c r="A13" s="19" t="n"/>
       <c r="B13" s="18" t="n"/>
       <c r="C13" s="18" t="n"/>
       <c r="D13" s="18" t="n"/>
-      <c r="E13" s="18" t="n"/>
+      <c r="E13" s="19" t="n"/>
       <c r="F13" s="18" t="n"/>
-      <c r="G13" s="18" t="n"/>
+      <c r="G13" s="27">
+        <f>IF(A13="","",WORKDAY(A13,-2))</f>
+        <v/>
+      </c>
       <c r="H13" s="18" t="n"/>
       <c r="I13" s="18" t="n"/>
       <c r="J13" s="18" t="n"/>
+      <c r="K13" s="18" t="n"/>
+      <c r="L13" s="18" t="n"/>
+      <c r="M13" s="18" t="n"/>
+      <c r="N13" s="18" t="n"/>
+      <c r="O13" s="18" t="n"/>
     </row>
     <row r="14" ht="36" customHeight="1">
       <c r="A14" s="23" t="n"/>
       <c r="B14" s="22" t="n"/>
       <c r="C14" s="22" t="n"/>
       <c r="D14" s="22" t="n"/>
-      <c r="E14" s="22" t="n"/>
+      <c r="E14" s="23" t="n"/>
       <c r="F14" s="22" t="n"/>
-      <c r="G14" s="22" t="n"/>
+      <c r="G14" s="27">
+        <f>IF(A14="","",WORKDAY(A14,-2))</f>
+        <v/>
+      </c>
       <c r="H14" s="22" t="n"/>
       <c r="I14" s="22" t="n"/>
       <c r="J14" s="22" t="n"/>
+      <c r="K14" s="22" t="n"/>
+      <c r="L14" s="22" t="n"/>
+      <c r="M14" s="22" t="n"/>
+      <c r="N14" s="22" t="n"/>
+      <c r="O14" s="22" t="n"/>
     </row>
     <row r="15" ht="36" customHeight="1">
       <c r="A15" s="19" t="n"/>
       <c r="B15" s="18" t="n"/>
       <c r="C15" s="18" t="n"/>
       <c r="D15" s="18" t="n"/>
-      <c r="E15" s="18" t="n"/>
+      <c r="E15" s="19" t="n"/>
       <c r="F15" s="18" t="n"/>
-      <c r="G15" s="18" t="n"/>
+      <c r="G15" s="27">
+        <f>IF(A15="","",WORKDAY(A15,-2))</f>
+        <v/>
+      </c>
       <c r="H15" s="18" t="n"/>
       <c r="I15" s="18" t="n"/>
       <c r="J15" s="18" t="n"/>
+      <c r="K15" s="18" t="n"/>
+      <c r="L15" s="18" t="n"/>
+      <c r="M15" s="18" t="n"/>
+      <c r="N15" s="18" t="n"/>
+      <c r="O15" s="18" t="n"/>
     </row>
     <row r="16" ht="36" customHeight="1">
       <c r="A16" s="23" t="n"/>
       <c r="B16" s="22" t="n"/>
       <c r="C16" s="22" t="n"/>
       <c r="D16" s="22" t="n"/>
-      <c r="E16" s="22" t="n"/>
+      <c r="E16" s="23" t="n"/>
       <c r="F16" s="22" t="n"/>
-      <c r="G16" s="22" t="n"/>
+      <c r="G16" s="27">
+        <f>IF(A16="","",WORKDAY(A16,-2))</f>
+        <v/>
+      </c>
       <c r="H16" s="22" t="n"/>
       <c r="I16" s="22" t="n"/>
       <c r="J16" s="22" t="n"/>
+      <c r="K16" s="22" t="n"/>
+      <c r="L16" s="22" t="n"/>
+      <c r="M16" s="22" t="n"/>
+      <c r="N16" s="22" t="n"/>
+      <c r="O16" s="22" t="n"/>
     </row>
     <row r="17" ht="36" customHeight="1">
       <c r="A17" s="19" t="n"/>
       <c r="B17" s="18" t="n"/>
       <c r="C17" s="18" t="n"/>
       <c r="D17" s="18" t="n"/>
-      <c r="E17" s="18" t="n"/>
+      <c r="E17" s="19" t="n"/>
       <c r="F17" s="18" t="n"/>
-      <c r="G17" s="18" t="n"/>
+      <c r="G17" s="27">
+        <f>IF(A17="","",WORKDAY(A17,-2))</f>
+        <v/>
+      </c>
       <c r="H17" s="18" t="n"/>
       <c r="I17" s="18" t="n"/>
       <c r="J17" s="18" t="n"/>
+      <c r="K17" s="18" t="n"/>
+      <c r="L17" s="18" t="n"/>
+      <c r="M17" s="18" t="n"/>
+      <c r="N17" s="18" t="n"/>
+      <c r="O17" s="18" t="n"/>
     </row>
     <row r="18" ht="36" customHeight="1">
       <c r="A18" s="23" t="n"/>
       <c r="B18" s="22" t="n"/>
       <c r="C18" s="22" t="n"/>
       <c r="D18" s="22" t="n"/>
-      <c r="E18" s="22" t="n"/>
+      <c r="E18" s="23" t="n"/>
       <c r="F18" s="22" t="n"/>
-      <c r="G18" s="22" t="n"/>
+      <c r="G18" s="27">
+        <f>IF(A18="","",WORKDAY(A18,-2))</f>
+        <v/>
+      </c>
       <c r="H18" s="22" t="n"/>
       <c r="I18" s="22" t="n"/>
       <c r="J18" s="22" t="n"/>
+      <c r="K18" s="22" t="n"/>
+      <c r="L18" s="22" t="n"/>
+      <c r="M18" s="22" t="n"/>
+      <c r="N18" s="22" t="n"/>
+      <c r="O18" s="22" t="n"/>
     </row>
     <row r="19" ht="36" customHeight="1">
       <c r="A19" s="19" t="n"/>
       <c r="B19" s="18" t="n"/>
       <c r="C19" s="18" t="n"/>
       <c r="D19" s="18" t="n"/>
-      <c r="E19" s="18" t="n"/>
+      <c r="E19" s="19" t="n"/>
       <c r="F19" s="18" t="n"/>
-      <c r="G19" s="18" t="n"/>
+      <c r="G19" s="27">
+        <f>IF(A19="","",WORKDAY(A19,-2))</f>
+        <v/>
+      </c>
       <c r="H19" s="18" t="n"/>
       <c r="I19" s="18" t="n"/>
       <c r="J19" s="18" t="n"/>
+      <c r="K19" s="18" t="n"/>
+      <c r="L19" s="18" t="n"/>
+      <c r="M19" s="18" t="n"/>
+      <c r="N19" s="18" t="n"/>
+      <c r="O19" s="18" t="n"/>
     </row>
     <row r="20" ht="36" customHeight="1">
       <c r="A20" s="23" t="n"/>
       <c r="B20" s="22" t="n"/>
       <c r="C20" s="22" t="n"/>
       <c r="D20" s="22" t="n"/>
-      <c r="E20" s="22" t="n"/>
+      <c r="E20" s="23" t="n"/>
       <c r="F20" s="22" t="n"/>
-      <c r="G20" s="22" t="n"/>
+      <c r="G20" s="27">
+        <f>IF(A20="","",WORKDAY(A20,-2))</f>
+        <v/>
+      </c>
       <c r="H20" s="22" t="n"/>
       <c r="I20" s="22" t="n"/>
       <c r="J20" s="22" t="n"/>
+      <c r="K20" s="22" t="n"/>
+      <c r="L20" s="22" t="n"/>
+      <c r="M20" s="22" t="n"/>
+      <c r="N20" s="22" t="n"/>
+      <c r="O20" s="22" t="n"/>
     </row>
     <row r="21" ht="36" customHeight="1">
       <c r="A21" s="19" t="n"/>
       <c r="B21" s="18" t="n"/>
       <c r="C21" s="18" t="n"/>
       <c r="D21" s="18" t="n"/>
-      <c r="E21" s="18" t="n"/>
+      <c r="E21" s="19" t="n"/>
       <c r="F21" s="18" t="n"/>
-      <c r="G21" s="18" t="n"/>
+      <c r="G21" s="27">
+        <f>IF(A21="","",WORKDAY(A21,-2))</f>
+        <v/>
+      </c>
       <c r="H21" s="18" t="n"/>
       <c r="I21" s="18" t="n"/>
       <c r="J21" s="18" t="n"/>
+      <c r="K21" s="18" t="n"/>
+      <c r="L21" s="18" t="n"/>
+      <c r="M21" s="18" t="n"/>
+      <c r="N21" s="18" t="n"/>
+      <c r="O21" s="18" t="n"/>
     </row>
     <row r="22" ht="36" customHeight="1">
       <c r="A22" s="23" t="n"/>
       <c r="B22" s="22" t="n"/>
       <c r="C22" s="22" t="n"/>
       <c r="D22" s="22" t="n"/>
-      <c r="E22" s="22" t="n"/>
+      <c r="E22" s="23" t="n"/>
       <c r="F22" s="22" t="n"/>
-      <c r="G22" s="22" t="n"/>
+      <c r="G22" s="27">
+        <f>IF(A22="","",WORKDAY(A22,-2))</f>
+        <v/>
+      </c>
       <c r="H22" s="22" t="n"/>
       <c r="I22" s="22" t="n"/>
       <c r="J22" s="22" t="n"/>
+      <c r="K22" s="22" t="n"/>
+      <c r="L22" s="22" t="n"/>
+      <c r="M22" s="22" t="n"/>
+      <c r="N22" s="22" t="n"/>
+      <c r="O22" s="22" t="n"/>
     </row>
     <row r="23" ht="36" customHeight="1">
       <c r="A23" s="19" t="n"/>
       <c r="B23" s="18" t="n"/>
       <c r="C23" s="18" t="n"/>
       <c r="D23" s="18" t="n"/>
-      <c r="E23" s="18" t="n"/>
+      <c r="E23" s="19" t="n"/>
       <c r="F23" s="18" t="n"/>
-      <c r="G23" s="18" t="n"/>
+      <c r="G23" s="27">
+        <f>IF(A23="","",WORKDAY(A23,-2))</f>
+        <v/>
+      </c>
       <c r="H23" s="18" t="n"/>
       <c r="I23" s="18" t="n"/>
       <c r="J23" s="18" t="n"/>
+      <c r="K23" s="18" t="n"/>
+      <c r="L23" s="18" t="n"/>
+      <c r="M23" s="18" t="n"/>
+      <c r="N23" s="18" t="n"/>
+      <c r="O23" s="18" t="n"/>
     </row>
     <row r="24" ht="36" customHeight="1">
       <c r="A24" s="23" t="n"/>
       <c r="B24" s="22" t="n"/>
       <c r="C24" s="22" t="n"/>
       <c r="D24" s="22" t="n"/>
-      <c r="E24" s="22" t="n"/>
+      <c r="E24" s="23" t="n"/>
       <c r="F24" s="22" t="n"/>
-      <c r="G24" s="22" t="n"/>
+      <c r="G24" s="27">
+        <f>IF(A24="","",WORKDAY(A24,-2))</f>
+        <v/>
+      </c>
       <c r="H24" s="22" t="n"/>
       <c r="I24" s="22" t="n"/>
       <c r="J24" s="22" t="n"/>
+      <c r="K24" s="22" t="n"/>
+      <c r="L24" s="22" t="n"/>
+      <c r="M24" s="22" t="n"/>
+      <c r="N24" s="22" t="n"/>
+      <c r="O24" s="22" t="n"/>
     </row>
     <row r="25" ht="36" customHeight="1">
       <c r="A25" s="19" t="n"/>
       <c r="B25" s="18" t="n"/>
       <c r="C25" s="18" t="n"/>
       <c r="D25" s="18" t="n"/>
-      <c r="E25" s="18" t="n"/>
+      <c r="E25" s="19" t="n"/>
       <c r="F25" s="18" t="n"/>
-      <c r="G25" s="18" t="n"/>
+      <c r="G25" s="27">
+        <f>IF(A25="","",WORKDAY(A25,-2))</f>
+        <v/>
+      </c>
       <c r="H25" s="18" t="n"/>
       <c r="I25" s="18" t="n"/>
       <c r="J25" s="18" t="n"/>
+      <c r="K25" s="18" t="n"/>
+      <c r="L25" s="18" t="n"/>
+      <c r="M25" s="18" t="n"/>
+      <c r="N25" s="18" t="n"/>
+      <c r="O25" s="18" t="n"/>
     </row>
     <row r="26" ht="36" customHeight="1">
       <c r="A26" s="23" t="n"/>
       <c r="B26" s="22" t="n"/>
       <c r="C26" s="22" t="n"/>
       <c r="D26" s="22" t="n"/>
-      <c r="E26" s="22" t="n"/>
+      <c r="E26" s="23" t="n"/>
       <c r="F26" s="22" t="n"/>
-      <c r="G26" s="22" t="n"/>
+      <c r="G26" s="27">
+        <f>IF(A26="","",WORKDAY(A26,-2))</f>
+        <v/>
+      </c>
       <c r="H26" s="22" t="n"/>
       <c r="I26" s="22" t="n"/>
       <c r="J26" s="22" t="n"/>
+      <c r="K26" s="22" t="n"/>
+      <c r="L26" s="22" t="n"/>
+      <c r="M26" s="22" t="n"/>
+      <c r="N26" s="22" t="n"/>
+      <c r="O26" s="22" t="n"/>
     </row>
     <row r="27" ht="36" customHeight="1">
       <c r="A27" s="19" t="n"/>
       <c r="B27" s="18" t="n"/>
       <c r="C27" s="18" t="n"/>
       <c r="D27" s="18" t="n"/>
-      <c r="E27" s="18" t="n"/>
+      <c r="E27" s="19" t="n"/>
       <c r="F27" s="18" t="n"/>
-      <c r="G27" s="18" t="n"/>
+      <c r="G27" s="27">
+        <f>IF(A27="","",WORKDAY(A27,-2))</f>
+        <v/>
+      </c>
       <c r="H27" s="18" t="n"/>
       <c r="I27" s="18" t="n"/>
       <c r="J27" s="18" t="n"/>
+      <c r="K27" s="18" t="n"/>
+      <c r="L27" s="18" t="n"/>
+      <c r="M27" s="18" t="n"/>
+      <c r="N27" s="18" t="n"/>
+      <c r="O27" s="18" t="n"/>
     </row>
     <row r="28" ht="36" customHeight="1">
       <c r="A28" s="23" t="n"/>
       <c r="B28" s="22" t="n"/>
       <c r="C28" s="22" t="n"/>
       <c r="D28" s="22" t="n"/>
-      <c r="E28" s="22" t="n"/>
+      <c r="E28" s="23" t="n"/>
       <c r="F28" s="22" t="n"/>
-      <c r="G28" s="22" t="n"/>
+      <c r="G28" s="27">
+        <f>IF(A28="","",WORKDAY(A28,-2))</f>
+        <v/>
+      </c>
       <c r="H28" s="22" t="n"/>
       <c r="I28" s="22" t="n"/>
       <c r="J28" s="22" t="n"/>
+      <c r="K28" s="22" t="n"/>
+      <c r="L28" s="22" t="n"/>
+      <c r="M28" s="22" t="n"/>
+      <c r="N28" s="22" t="n"/>
+      <c r="O28" s="22" t="n"/>
     </row>
     <row r="29" ht="36" customHeight="1">
       <c r="A29" s="19" t="n"/>
       <c r="B29" s="18" t="n"/>
       <c r="C29" s="18" t="n"/>
       <c r="D29" s="18" t="n"/>
-      <c r="E29" s="18" t="n"/>
+      <c r="E29" s="19" t="n"/>
       <c r="F29" s="18" t="n"/>
-      <c r="G29" s="18" t="n"/>
+      <c r="G29" s="27">
+        <f>IF(A29="","",WORKDAY(A29,-2))</f>
+        <v/>
+      </c>
       <c r="H29" s="18" t="n"/>
       <c r="I29" s="18" t="n"/>
       <c r="J29" s="18" t="n"/>
+      <c r="K29" s="18" t="n"/>
+      <c r="L29" s="18" t="n"/>
+      <c r="M29" s="18" t="n"/>
+      <c r="N29" s="18" t="n"/>
+      <c r="O29" s="18" t="n"/>
     </row>
     <row r="30" ht="36" customHeight="1">
       <c r="A30" s="23" t="n"/>
       <c r="B30" s="22" t="n"/>
       <c r="C30" s="22" t="n"/>
       <c r="D30" s="22" t="n"/>
-      <c r="E30" s="22" t="n"/>
+      <c r="E30" s="23" t="n"/>
       <c r="F30" s="22" t="n"/>
-      <c r="G30" s="22" t="n"/>
+      <c r="G30" s="27">
+        <f>IF(A30="","",WORKDAY(A30,-2))</f>
+        <v/>
+      </c>
       <c r="H30" s="22" t="n"/>
       <c r="I30" s="22" t="n"/>
       <c r="J30" s="22" t="n"/>
+      <c r="K30" s="22" t="n"/>
+      <c r="L30" s="22" t="n"/>
+      <c r="M30" s="22" t="n"/>
+      <c r="N30" s="22" t="n"/>
+      <c r="O30" s="22" t="n"/>
     </row>
     <row r="31" ht="36" customHeight="1">
       <c r="A31" s="19" t="n"/>
       <c r="B31" s="18" t="n"/>
       <c r="C31" s="18" t="n"/>
       <c r="D31" s="18" t="n"/>
-      <c r="E31" s="18" t="n"/>
+      <c r="E31" s="19" t="n"/>
       <c r="F31" s="18" t="n"/>
-      <c r="G31" s="18" t="n"/>
+      <c r="G31" s="27">
+        <f>IF(A31="","",WORKDAY(A31,-2))</f>
+        <v/>
+      </c>
       <c r="H31" s="18" t="n"/>
       <c r="I31" s="18" t="n"/>
       <c r="J31" s="18" t="n"/>
+      <c r="K31" s="18" t="n"/>
+      <c r="L31" s="18" t="n"/>
+      <c r="M31" s="18" t="n"/>
+      <c r="N31" s="18" t="n"/>
+      <c r="O31" s="18" t="n"/>
     </row>
     <row r="32" ht="36" customHeight="1">
       <c r="A32" s="23" t="n"/>
       <c r="B32" s="22" t="n"/>
       <c r="C32" s="22" t="n"/>
       <c r="D32" s="22" t="n"/>
-      <c r="E32" s="22" t="n"/>
+      <c r="E32" s="23" t="n"/>
       <c r="F32" s="22" t="n"/>
-      <c r="G32" s="22" t="n"/>
+      <c r="G32" s="27">
+        <f>IF(A32="","",WORKDAY(A32,-2))</f>
+        <v/>
+      </c>
       <c r="H32" s="22" t="n"/>
       <c r="I32" s="22" t="n"/>
       <c r="J32" s="22" t="n"/>
+      <c r="K32" s="22" t="n"/>
+      <c r="L32" s="22" t="n"/>
+      <c r="M32" s="22" t="n"/>
+      <c r="N32" s="22" t="n"/>
+      <c r="O32" s="22" t="n"/>
     </row>
     <row r="33" ht="36" customHeight="1">
       <c r="A33" s="19" t="n"/>
       <c r="B33" s="18" t="n"/>
       <c r="C33" s="18" t="n"/>
       <c r="D33" s="18" t="n"/>
-      <c r="E33" s="18" t="n"/>
+      <c r="E33" s="19" t="n"/>
       <c r="F33" s="18" t="n"/>
-      <c r="G33" s="18" t="n"/>
+      <c r="G33" s="27">
+        <f>IF(A33="","",WORKDAY(A33,-2))</f>
+        <v/>
+      </c>
       <c r="H33" s="18" t="n"/>
       <c r="I33" s="18" t="n"/>
       <c r="J33" s="18" t="n"/>
+      <c r="K33" s="18" t="n"/>
+      <c r="L33" s="18" t="n"/>
+      <c r="M33" s="18" t="n"/>
+      <c r="N33" s="18" t="n"/>
+      <c r="O33" s="18" t="n"/>
     </row>
     <row r="34" ht="36" customHeight="1">
       <c r="A34" s="23" t="n"/>
       <c r="B34" s="22" t="n"/>
       <c r="C34" s="22" t="n"/>
       <c r="D34" s="22" t="n"/>
-      <c r="E34" s="22" t="n"/>
+      <c r="E34" s="23" t="n"/>
       <c r="F34" s="22" t="n"/>
-      <c r="G34" s="22" t="n"/>
+      <c r="G34" s="27">
+        <f>IF(A34="","",WORKDAY(A34,-2))</f>
+        <v/>
+      </c>
       <c r="H34" s="22" t="n"/>
       <c r="I34" s="22" t="n"/>
       <c r="J34" s="22" t="n"/>
+      <c r="K34" s="22" t="n"/>
+      <c r="L34" s="22" t="n"/>
+      <c r="M34" s="22" t="n"/>
+      <c r="N34" s="22" t="n"/>
+      <c r="O34" s="22" t="n"/>
     </row>
     <row r="35" ht="36" customHeight="1">
       <c r="A35" s="19" t="n"/>
       <c r="B35" s="18" t="n"/>
       <c r="C35" s="18" t="n"/>
       <c r="D35" s="18" t="n"/>
-      <c r="E35" s="18" t="n"/>
+      <c r="E35" s="19" t="n"/>
       <c r="F35" s="18" t="n"/>
-      <c r="G35" s="18" t="n"/>
+      <c r="G35" s="27">
+        <f>IF(A35="","",WORKDAY(A35,-2))</f>
+        <v/>
+      </c>
       <c r="H35" s="18" t="n"/>
       <c r="I35" s="18" t="n"/>
       <c r="J35" s="18" t="n"/>
+      <c r="K35" s="18" t="n"/>
+      <c r="L35" s="18" t="n"/>
+      <c r="M35" s="18" t="n"/>
+      <c r="N35" s="18" t="n"/>
+      <c r="O35" s="18" t="n"/>
     </row>
     <row r="36" ht="36" customHeight="1">
       <c r="A36" s="23" t="n"/>
       <c r="B36" s="22" t="n"/>
       <c r="C36" s="22" t="n"/>
       <c r="D36" s="22" t="n"/>
-      <c r="E36" s="22" t="n"/>
+      <c r="E36" s="23" t="n"/>
       <c r="F36" s="22" t="n"/>
-      <c r="G36" s="22" t="n"/>
+      <c r="G36" s="27">
+        <f>IF(A36="","",WORKDAY(A36,-2))</f>
+        <v/>
+      </c>
       <c r="H36" s="22" t="n"/>
       <c r="I36" s="22" t="n"/>
       <c r="J36" s="22" t="n"/>
+      <c r="K36" s="22" t="n"/>
+      <c r="L36" s="22" t="n"/>
+      <c r="M36" s="22" t="n"/>
+      <c r="N36" s="22" t="n"/>
+      <c r="O36" s="22" t="n"/>
     </row>
     <row r="37" ht="36" customHeight="1">
       <c r="A37" s="19" t="n"/>
       <c r="B37" s="18" t="n"/>
       <c r="C37" s="18" t="n"/>
       <c r="D37" s="18" t="n"/>
-      <c r="E37" s="18" t="n"/>
+      <c r="E37" s="19" t="n"/>
       <c r="F37" s="18" t="n"/>
-      <c r="G37" s="18" t="n"/>
+      <c r="G37" s="27">
+        <f>IF(A37="","",WORKDAY(A37,-2))</f>
+        <v/>
+      </c>
       <c r="H37" s="18" t="n"/>
       <c r="I37" s="18" t="n"/>
       <c r="J37" s="18" t="n"/>
+      <c r="K37" s="18" t="n"/>
+      <c r="L37" s="18" t="n"/>
+      <c r="M37" s="18" t="n"/>
+      <c r="N37" s="18" t="n"/>
+      <c r="O37" s="18" t="n"/>
     </row>
     <row r="38" ht="36" customHeight="1">
       <c r="A38" s="23" t="n"/>
       <c r="B38" s="22" t="n"/>
       <c r="C38" s="22" t="n"/>
       <c r="D38" s="22" t="n"/>
-      <c r="E38" s="22" t="n"/>
+      <c r="E38" s="23" t="n"/>
       <c r="F38" s="22" t="n"/>
-      <c r="G38" s="22" t="n"/>
+      <c r="G38" s="27">
+        <f>IF(A38="","",WORKDAY(A38,-2))</f>
+        <v/>
+      </c>
       <c r="H38" s="22" t="n"/>
       <c r="I38" s="22" t="n"/>
       <c r="J38" s="22" t="n"/>
+      <c r="K38" s="22" t="n"/>
+      <c r="L38" s="22" t="n"/>
+      <c r="M38" s="22" t="n"/>
+      <c r="N38" s="22" t="n"/>
+      <c r="O38" s="22" t="n"/>
     </row>
     <row r="39" ht="36" customHeight="1">
       <c r="A39" s="19" t="n"/>
       <c r="B39" s="18" t="n"/>
       <c r="C39" s="18" t="n"/>
       <c r="D39" s="18" t="n"/>
-      <c r="E39" s="18" t="n"/>
+      <c r="E39" s="19" t="n"/>
       <c r="F39" s="18" t="n"/>
-      <c r="G39" s="18" t="n"/>
+      <c r="G39" s="27">
+        <f>IF(A39="","",WORKDAY(A39,-2))</f>
+        <v/>
+      </c>
       <c r="H39" s="18" t="n"/>
       <c r="I39" s="18" t="n"/>
       <c r="J39" s="18" t="n"/>
+      <c r="K39" s="18" t="n"/>
+      <c r="L39" s="18" t="n"/>
+      <c r="M39" s="18" t="n"/>
+      <c r="N39" s="18" t="n"/>
+      <c r="O39" s="18" t="n"/>
     </row>
     <row r="40" ht="36" customHeight="1">
       <c r="A40" s="23" t="n"/>
       <c r="B40" s="22" t="n"/>
       <c r="C40" s="22" t="n"/>
       <c r="D40" s="22" t="n"/>
-      <c r="E40" s="22" t="n"/>
+      <c r="E40" s="23" t="n"/>
       <c r="F40" s="22" t="n"/>
-      <c r="G40" s="22" t="n"/>
+      <c r="G40" s="27">
+        <f>IF(A40="","",WORKDAY(A40,-2))</f>
+        <v/>
+      </c>
       <c r="H40" s="22" t="n"/>
       <c r="I40" s="22" t="n"/>
       <c r="J40" s="22" t="n"/>
+      <c r="K40" s="22" t="n"/>
+      <c r="L40" s="22" t="n"/>
+      <c r="M40" s="22" t="n"/>
+      <c r="N40" s="22" t="n"/>
+      <c r="O40" s="22" t="n"/>
     </row>
     <row r="41" ht="36" customHeight="1">
       <c r="A41" s="19" t="n"/>
       <c r="B41" s="18" t="n"/>
       <c r="C41" s="18" t="n"/>
       <c r="D41" s="18" t="n"/>
-      <c r="E41" s="18" t="n"/>
+      <c r="E41" s="19" t="n"/>
       <c r="F41" s="18" t="n"/>
-      <c r="G41" s="18" t="n"/>
+      <c r="G41" s="27">
+        <f>IF(A41="","",WORKDAY(A41,-2))</f>
+        <v/>
+      </c>
       <c r="H41" s="18" t="n"/>
       <c r="I41" s="18" t="n"/>
       <c r="J41" s="18" t="n"/>
+      <c r="K41" s="18" t="n"/>
+      <c r="L41" s="18" t="n"/>
+      <c r="M41" s="18" t="n"/>
+      <c r="N41" s="18" t="n"/>
+      <c r="O41" s="18" t="n"/>
     </row>
     <row r="42" ht="36" customHeight="1">
       <c r="A42" s="23" t="n"/>
       <c r="B42" s="22" t="n"/>
       <c r="C42" s="22" t="n"/>
       <c r="D42" s="22" t="n"/>
-      <c r="E42" s="22" t="n"/>
+      <c r="E42" s="23" t="n"/>
       <c r="F42" s="22" t="n"/>
-      <c r="G42" s="22" t="n"/>
+      <c r="G42" s="27">
+        <f>IF(A42="","",WORKDAY(A42,-2))</f>
+        <v/>
+      </c>
       <c r="H42" s="22" t="n"/>
       <c r="I42" s="22" t="n"/>
       <c r="J42" s="22" t="n"/>
+      <c r="K42" s="22" t="n"/>
+      <c r="L42" s="22" t="n"/>
+      <c r="M42" s="22" t="n"/>
+      <c r="N42" s="22" t="n"/>
+      <c r="O42" s="22" t="n"/>
     </row>
     <row r="43" ht="36" customHeight="1">
       <c r="A43" s="19" t="n"/>
       <c r="B43" s="18" t="n"/>
       <c r="C43" s="18" t="n"/>
       <c r="D43" s="18" t="n"/>
-      <c r="E43" s="18" t="n"/>
+      <c r="E43" s="19" t="n"/>
       <c r="F43" s="18" t="n"/>
-      <c r="G43" s="18" t="n"/>
+      <c r="G43" s="27">
+        <f>IF(A43="","",WORKDAY(A43,-2))</f>
+        <v/>
+      </c>
       <c r="H43" s="18" t="n"/>
       <c r="I43" s="18" t="n"/>
       <c r="J43" s="18" t="n"/>
+      <c r="K43" s="18" t="n"/>
+      <c r="L43" s="18" t="n"/>
+      <c r="M43" s="18" t="n"/>
+      <c r="N43" s="18" t="n"/>
+      <c r="O43" s="18" t="n"/>
     </row>
     <row r="44" ht="36" customHeight="1">
       <c r="A44" s="23" t="n"/>
       <c r="B44" s="22" t="n"/>
       <c r="C44" s="22" t="n"/>
       <c r="D44" s="22" t="n"/>
-      <c r="E44" s="22" t="n"/>
+      <c r="E44" s="23" t="n"/>
       <c r="F44" s="22" t="n"/>
-      <c r="G44" s="22" t="n"/>
+      <c r="G44" s="27">
+        <f>IF(A44="","",WORKDAY(A44,-2))</f>
+        <v/>
+      </c>
       <c r="H44" s="22" t="n"/>
       <c r="I44" s="22" t="n"/>
       <c r="J44" s="22" t="n"/>
+      <c r="K44" s="22" t="n"/>
+      <c r="L44" s="22" t="n"/>
+      <c r="M44" s="22" t="n"/>
+      <c r="N44" s="22" t="n"/>
+      <c r="O44" s="22" t="n"/>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="G5:G44">
+    <cfRule type="expression" priority="1" dxfId="2">
+      <formula>AND(ISNUMBER(G5),G5-TODAY()&gt;=0,G5-TODAY()&lt;=3)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="2">
+    <dataValidation sqref="D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D35 D36 D37 D38 D39 D40 D41 D42 D43 D44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"U (72 ore),B (10 giorni),D (30/60 giorni),P (120 giorni),Controllo,Privata"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H5 H6 H7 H8 H9 H10 H11 H12 H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H25 H26 H27 H28 H29 H30 H31 H32 H33 H34 H35 H36 H37 H38 H39 H40 H41 H42 H43 H44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Da pagare,Pagato,Esente,Privata"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
@@ -3651,37 +4279,37 @@
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="27" t="inlineStr">
+      <c r="B4" s="28" t="inlineStr">
         <is>
           <t>Lunedì</t>
         </is>
       </c>
-      <c r="C4" s="27" t="inlineStr">
+      <c r="C4" s="28" t="inlineStr">
         <is>
           <t>Martedì</t>
         </is>
       </c>
-      <c r="D4" s="27" t="inlineStr">
+      <c r="D4" s="28" t="inlineStr">
         <is>
           <t>Mercoledì</t>
         </is>
       </c>
-      <c r="E4" s="27" t="inlineStr">
+      <c r="E4" s="28" t="inlineStr">
         <is>
           <t>Giovedì</t>
         </is>
       </c>
-      <c r="F4" s="27" t="inlineStr">
+      <c r="F4" s="28" t="inlineStr">
         <is>
           <t>Venerdì</t>
         </is>
       </c>
-      <c r="G4" s="27" t="inlineStr">
+      <c r="G4" s="28" t="inlineStr">
         <is>
           <t>Sabato</t>
         </is>
       </c>
-      <c r="H4" s="27" t="inlineStr">
+      <c r="H4" s="28" t="inlineStr">
         <is>
           <t>Domenica</t>
         </is>
@@ -3693,17 +4321,17 @@
           <t>Mattina</t>
         </is>
       </c>
-      <c r="B5" s="28" t="inlineStr">
+      <c r="B5" s="29" t="inlineStr">
         <is>
           <t>Nido 8:30</t>
         </is>
       </c>
-      <c r="C5" s="28" t="n"/>
-      <c r="D5" s="28" t="n"/>
-      <c r="E5" s="28" t="n"/>
-      <c r="F5" s="28" t="n"/>
-      <c r="G5" s="28" t="n"/>
-      <c r="H5" s="28" t="n"/>
+      <c r="C5" s="29" t="n"/>
+      <c r="D5" s="29" t="n"/>
+      <c r="E5" s="29" t="n"/>
+      <c r="F5" s="29" t="n"/>
+      <c r="G5" s="29" t="n"/>
+      <c r="H5" s="29" t="n"/>
     </row>
     <row r="6" ht="48" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
@@ -3711,13 +4339,13 @@
           <t>Pomeriggio</t>
         </is>
       </c>
-      <c r="B6" s="29" t="n"/>
-      <c r="C6" s="29" t="n"/>
-      <c r="D6" s="29" t="n"/>
-      <c r="E6" s="29" t="n"/>
-      <c r="F6" s="29" t="n"/>
-      <c r="G6" s="29" t="n"/>
-      <c r="H6" s="29" t="n"/>
+      <c r="B6" s="30" t="n"/>
+      <c r="C6" s="30" t="n"/>
+      <c r="D6" s="30" t="n"/>
+      <c r="E6" s="30" t="n"/>
+      <c r="F6" s="30" t="n"/>
+      <c r="G6" s="30" t="n"/>
+      <c r="H6" s="30" t="n"/>
     </row>
     <row r="7" ht="48" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
@@ -3725,17 +4353,17 @@
           <t>Sera</t>
         </is>
       </c>
-      <c r="B7" s="28" t="inlineStr">
+      <c r="B7" s="29" t="inlineStr">
         <is>
           <t>Bagnetto, storia, nanna 20:30</t>
         </is>
       </c>
-      <c r="C7" s="28" t="n"/>
-      <c r="D7" s="28" t="n"/>
-      <c r="E7" s="28" t="n"/>
-      <c r="F7" s="28" t="n"/>
-      <c r="G7" s="28" t="n"/>
-      <c r="H7" s="28" t="n"/>
+      <c r="C7" s="29" t="n"/>
+      <c r="D7" s="29" t="n"/>
+      <c r="E7" s="29" t="n"/>
+      <c r="F7" s="29" t="n"/>
+      <c r="G7" s="29" t="n"/>
+      <c r="H7" s="29" t="n"/>
     </row>
     <row r="8" ht="48" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
@@ -3743,17 +4371,17 @@
           <t>Chi se ne occupa</t>
         </is>
       </c>
-      <c r="B8" s="29" t="inlineStr">
+      <c r="B8" s="30" t="inlineStr">
         <is>
           <t>Mamma mattina · Papà sera</t>
         </is>
       </c>
-      <c r="C8" s="29" t="n"/>
-      <c r="D8" s="29" t="n"/>
-      <c r="E8" s="29" t="n"/>
-      <c r="F8" s="29" t="n"/>
-      <c r="G8" s="29" t="n"/>
-      <c r="H8" s="29" t="n"/>
+      <c r="C8" s="30" t="n"/>
+      <c r="D8" s="30" t="n"/>
+      <c r="E8" s="30" t="n"/>
+      <c r="F8" s="30" t="n"/>
+      <c r="G8" s="30" t="n"/>
+      <c r="H8" s="30" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="13" t="inlineStr">
@@ -3876,18 +4504,46 @@
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="18" t="n"/>
-      <c r="B7" s="18" t="n"/>
-      <c r="C7" s="18" t="n"/>
-      <c r="D7" s="18" t="n"/>
-      <c r="E7" s="18" t="n"/>
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>CUP (prenotazioni)</t>
+        </is>
+      </c>
+      <c r="B7" s="18" t="inlineStr">
+        <is>
+          <t>CUP regionale</t>
+        </is>
+      </c>
+      <c r="C7" s="18" t="inlineStr"/>
+      <c r="D7" s="18" t="inlineStr">
+        <is>
+          <t>Per prenotare e disdire; segna anche sito e app</t>
+        </is>
+      </c>
+      <c r="E7" s="21" t="inlineStr">
+        <is>
+          <t>Cerca il numero della tua Regione</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="22" t="n"/>
-      <c r="B8" s="22" t="n"/>
-      <c r="C8" s="22" t="n"/>
-      <c r="D8" s="22" t="n"/>
-      <c r="E8" s="22" t="n"/>
+      <c r="A8" s="22" t="inlineStr">
+        <is>
+          <t>URP della ASL</t>
+        </is>
+      </c>
+      <c r="B8" s="22" t="inlineStr"/>
+      <c r="C8" s="22" t="inlineStr"/>
+      <c r="D8" s="22" t="inlineStr">
+        <is>
+          <t>Se la visita supera i tempi della ricetta</t>
+        </is>
+      </c>
+      <c r="E8" s="24" t="inlineStr">
+        <is>
+          <t>Cerca il numero della tua ASL</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="18" t="n"/>
@@ -4144,7 +4800,7 @@
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="A5 A6 A7 A8 A9 A10 A11 A12 A13 A14 A15 A16 A17 A18 A19 A20 A21 A22 A23 A24 A25 A26 A27 A28 A29 A30 A31 A32 A33 A34 A35 A36 A37 A38 A39 A40 A41 A42 A43 A44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Pediatra,Medico di famiglia,Guardia medica,ASL,Pronto soccorso,Nido / scuola,Nonni,Babysitter,Farmacia,Altro"</formula1>
+      <formula1>"Pediatra,Medico di famiglia,Guardia medica,CUP (prenotazioni),URP della ASL,Fascicolo sanitario (numero verde),Pronto soccorso,Nido / scuola,Nonni,Babysitter,Farmacia,Altro"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>